<commit_message>
budget working on all Qs! except still very slow.
</commit_message>
<xml_diff>
--- a/data/1038-0610-0614-day-larger-figures-test.xlsx
+++ b/data/1038-0610-0614-day-larger-figures-test.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://liveuclac-my.sharepoint.com/personal/ucabmr3_ucl_ac_uk/Documents/UCL_comp_sci/Sustainable_Systems_3/HP_Sus_Sys_3/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="21" documentId="8_{72E707BE-0160-4B47-9423-3E839962E439}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1EAF0E6C-2112-4DF4-9AF5-7B10343F1EEF}"/>
+  <xr:revisionPtr revIDLastSave="23" documentId="8_{72E707BE-0160-4B47-9423-3E839962E439}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{519346DE-E259-4608-AFAF-B4A35B4CF130}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="510" yWindow="4890" windowWidth="17670" windowHeight="9840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4095" yWindow="675" windowWidth="18825" windowHeight="8235" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="4" r:id="rId1"/>
@@ -1786,7 +1786,7 @@
         <v>89.690228174603106</v>
       </c>
       <c r="L7" s="20">
-        <v>79.132013670350801</v>
+        <v>89.132013670350801</v>
       </c>
       <c r="M7" s="20">
         <v>1</v>
@@ -2270,7 +2270,7 @@
         <v>9</v>
       </c>
       <c r="AT9" s="20">
-        <v>1.00461538461538</v>
+        <v>71.004615384615306</v>
       </c>
       <c r="AU9" s="20">
         <v>0</v>

</xml_diff>

<commit_message>
last test with smaller figures + working: works with Q2 on second run. others OK.
</commit_message>
<xml_diff>
--- a/data/1038-0610-0614-day-larger-figures-test.xlsx
+++ b/data/1038-0610-0614-day-larger-figures-test.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://liveuclac-my.sharepoint.com/personal/ucabmr3_ucl_ac_uk/Documents/UCL_comp_sci/Sustainable_Systems_3/HP_Sus_Sys_3/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="23" documentId="8_{72E707BE-0160-4B47-9423-3E839962E439}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{519346DE-E259-4608-AFAF-B4A35B4CF130}"/>
+  <xr:revisionPtr revIDLastSave="24" documentId="8_{72E707BE-0160-4B47-9423-3E839962E439}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A83EA49F-FD48-4F55-B28D-B1775F13EF54}"/>
   <bookViews>
-    <workbookView xWindow="4095" yWindow="675" windowWidth="18825" windowHeight="8235" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="630" yWindow="3390" windowWidth="18825" windowHeight="9510" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="4" r:id="rId1"/>
@@ -1880,7 +1880,7 @@
         <v>3</v>
       </c>
       <c r="AT7" s="20">
-        <v>17.543209999999998</v>
+        <v>13.54321</v>
       </c>
       <c r="AU7" s="20">
         <v>0</v>

</xml_diff>